<commit_message>
data(isobutanol): feedstock starch content uniform 0.684-0.743 (A workbook)
Same change as f4951a52, now for the scenario-A parameter-distribution
workbook (it was open in Excel then): 'Feedstock starch content'
Triangular 0.576 / 0.72 / 0.864 -> Uniform 0.684-0.743 kg/dry-kg, blank
Midpoint, Baseline 0.72 unchanged, References = U.S. Grains Council
2024/2025 Corn Harvest Quality Report, 2022-2024 min / max (dry basis).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
+++ b/biorefineries/isobutanol/analyses/full/parameter_distributions/parameter-distributions_corn_IBO_EtOH_A.xlsx
@@ -1136,19 +1136,21 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Triangular</t>
+          <t>Uniform</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.576</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>0.72</v>
-      </c>
+        <v>0.6840000000000001</v>
+      </c>
+      <c r="H15" s="3" t="n"/>
       <c r="I15" s="3" t="n">
-        <v>0.864</v>
-      </c>
-      <c r="J15" s="3" t="n"/>
+        <v>0.743</v>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Uniform over the min-max of the 2022-2024 U.S. corn starch content (dry basis) 68.4-74.3 %, U.S. Grains Council, 2024/2025 Corn Harvest Quality Report, https://grains.org/corn_report/corn-harvest-quality-report-2024-2025-2/</t>
+        </is>
+      </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
           <t>fixed_F_mass = feedstock.F_mass; feedstock.imass['Starch'] = x * (fixed_F_mass - feedstock.imass['Water']); feedstock.F_mass = fixed_F_mass</t>

</xml_diff>